<commit_message>
Improved Test Scenario and Complete the test cases of product page
</commit_message>
<xml_diff>
--- a/Project-2/TestCases_SauceDemo.xlsx
+++ b/Project-2/TestCases_SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d09b73bd954f8bef/GitHub-Backup/Manual-Testing-Projects/Project-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="8_{9932A3A6-EBCC-492E-807B-E0D10A0E8F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD6EB391-BBD4-49D5-8D34-14D6D656F45E}"/>
+  <xr:revisionPtr revIDLastSave="295" documentId="8_{9932A3A6-EBCC-492E-807B-E0D10A0E8F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EDBD1F5-8B4E-4A16-9129-CB6A2BA088D3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CC2F979-7099-4757-920D-883D45E7E350}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2CC2F979-7099-4757-920D-883D45E7E350}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="135">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -320,6 +320,217 @@
   </si>
   <si>
     <t>All the ui elements of login page like text, input field, button should be visibile</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_01</t>
+  </si>
+  <si>
+    <t>Verify product list is displalyed</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Observe the appeared product list</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>System should display product list in which all the product should be perfectly visible without any ui error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify user interface </t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Observe the product page</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_03</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_02</t>
+  </si>
+  <si>
+    <t>System should show correct product name</t>
+  </si>
+  <si>
+    <t>Verify product name detail</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_04</t>
+  </si>
+  <si>
+    <t>Verify product description detail</t>
+  </si>
+  <si>
+    <t>System should show correct product description</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_05</t>
+  </si>
+  <si>
+    <t>Verify product price detail</t>
+  </si>
+  <si>
+    <t>System should show correct product price</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_06</t>
+  </si>
+  <si>
+    <t>Verfiy product page redirection through image</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Click the image of any product from list
+4.Observe the appeared product page</t>
+  </si>
+  <si>
+    <t>System should redirect user to correct product page</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_07</t>
+  </si>
+  <si>
+    <t>Verfiy product page redirection through product name</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Click the name of any product from list
+4.Observe the appeared product page</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_08</t>
+  </si>
+  <si>
+    <t>Verify user can add product to cart</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Click add to cart button of any product card
+4.Observe the cart icon number</t>
+  </si>
+  <si>
+    <t>Cart icon number should properly increase on user add to cart action</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_09</t>
+  </si>
+  <si>
+    <t>Verify user can remove product from cart</t>
+  </si>
+  <si>
+    <t>Cart icon number should decrease on user remove action</t>
+  </si>
+  <si>
+    <t>System should not show any ui error and all the element should perfectly visible</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_10</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Click add to cart button of any product card
+4.Click remove button of added product
+5.Observe the cart icon number</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Observe the product list that are arranged in default filter order Name (A to Z)</t>
+  </si>
+  <si>
+    <t>System should show products in list according to Name (A to Z) filter order</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_11</t>
+  </si>
+  <si>
+    <t>Verify product sorting behaviour from filter option</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Choose option Name (Z to A) of filter filter
+4.Observe the product list</t>
+  </si>
+  <si>
+    <t>System should show products in list according to Name (Z to A) filter order</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_12</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Choose option Price (Low to High) of filter filter
+4.Observe the product list</t>
+  </si>
+  <si>
+    <t>System should show products in list according to Price (Low to High) filter order</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_13</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Choose option Price (High to Low) of filter filter
+4.Observe the product list</t>
+  </si>
+  <si>
+    <t>System should show products in list according to Price (High to Low) filter order</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_14</t>
+  </si>
+  <si>
+    <t>Verify prouct page logout button</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Click the navbar humburger button of product page
+4.Click logout option
+4.Observe the redirected page</t>
+  </si>
+  <si>
+    <t>System should redirect user to login page</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_15</t>
+  </si>
+  <si>
+    <t>Verify footer links</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Click any social media platform link from footer
+4.Observe redirected page</t>
+  </si>
+  <si>
+    <t>Sytem should redirect user to correct social platform</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_16</t>
+  </si>
+  <si>
+    <t>Verify user interface of product page</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Observe the text and content of footer</t>
+  </si>
+  <si>
+    <t>System should display footer content correctly</t>
   </si>
 </sst>
 </file>
@@ -391,12 +602,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -763,13 +971,13 @@
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="2"/>
@@ -782,13 +990,13 @@
       <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>16</v>
       </c>
       <c r="F3" s="2"/>
@@ -801,13 +1009,13 @@
       <c r="B4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="2"/>
@@ -820,13 +1028,13 @@
       <c r="B5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="F5" s="2"/>
@@ -836,16 +1044,16 @@
       <c r="A6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>28</v>
       </c>
       <c r="F6" s="2"/>
@@ -855,16 +1063,16 @@
       <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="2" t="s">
         <v>33</v>
       </c>
       <c r="F7" s="2"/>
@@ -874,16 +1082,16 @@
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="2" t="s">
         <v>33</v>
       </c>
       <c r="F8" s="2"/>
@@ -893,16 +1101,16 @@
       <c r="A9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="2" t="s">
         <v>42</v>
       </c>
       <c r="F9" s="2"/>
@@ -912,16 +1120,16 @@
       <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="2" t="s">
         <v>47</v>
       </c>
       <c r="F10" s="2"/>
@@ -931,16 +1139,16 @@
       <c r="A11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F11" s="2"/>
@@ -950,16 +1158,16 @@
       <c r="A12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="2" t="s">
         <v>57</v>
       </c>
       <c r="F12" s="2"/>
@@ -969,16 +1177,16 @@
       <c r="A13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="2" t="s">
         <v>62</v>
       </c>
       <c r="F13" s="2"/>
@@ -988,16 +1196,16 @@
       <c r="A14" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="2" t="s">
         <v>67</v>
       </c>
       <c r="F14" s="2"/>
@@ -1007,16 +1215,16 @@
       <c r="A15" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="2" t="s">
         <v>72</v>
       </c>
       <c r="F15" s="2"/>
@@ -1026,14 +1234,16 @@
       <c r="A16" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="4" t="s">
+      <c r="D16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>76</v>
       </c>
       <c r="F16" s="2"/>
@@ -1049,8 +1259,16 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -1074,6 +1292,310 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+    </row>
+    <row r="2" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:7" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:7" ht="156" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:7" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add: Complete and final test scenario and test case sheet
</commit_message>
<xml_diff>
--- a/Project-2/TestCases_SauceDemo.xlsx
+++ b/Project-2/TestCases_SauceDemo.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d09b73bd954f8bef/GitHub-Backup/Manual-Testing-Projects/Project-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="295" documentId="8_{9932A3A6-EBCC-492E-807B-E0D10A0E8F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EDBD1F5-8B4E-4A16-9129-CB6A2BA088D3}"/>
+  <xr:revisionPtr revIDLastSave="769" documentId="8_{9932A3A6-EBCC-492E-807B-E0D10A0E8F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{275953B8-B525-414F-9D96-44F200EE5628}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2CC2F979-7099-4757-920D-883D45E7E350}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{2CC2F979-7099-4757-920D-883D45E7E350}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Product" sheetId="2" r:id="rId2"/>
     <sheet name="Cart" sheetId="3" r:id="rId3"/>
-    <sheet name="Checkout" sheetId="4" r:id="rId4"/>
+    <sheet name="Checkout - Your Information" sheetId="4" r:id="rId4"/>
+    <sheet name="Checkout - Overview" sheetId="5" r:id="rId5"/>
+    <sheet name="Checkout - Complete" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="414">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -494,13 +496,6 @@
     <t>Verify prouct page logout button</t>
   </si>
   <si>
-    <t>1.Open saucedemo website
-2.Login with valid credential
-3.Click the navbar humburger button of product page
-4.Click logout option
-4.Observe the redirected page</t>
-  </si>
-  <si>
     <t>System should redirect user to login page</t>
   </si>
   <si>
@@ -531,13 +526,957 @@
   </si>
   <si>
     <t>System should display footer content correctly</t>
+  </si>
+  <si>
+    <t>TC_CART_01</t>
+  </si>
+  <si>
+    <t>Verify added products</t>
+  </si>
+  <si>
+    <t>TC_CART_02</t>
+  </si>
+  <si>
+    <t>Verify user interface</t>
+  </si>
+  <si>
+    <t>Cart label, qty, description, buttons color, section and all the ui alignment should be clear visible</t>
+  </si>
+  <si>
+    <t>TC_CART_03</t>
+  </si>
+  <si>
+    <t>TC_CART_04</t>
+  </si>
+  <si>
+    <t>TC_CART_05</t>
+  </si>
+  <si>
+    <t>TC_CART_06</t>
+  </si>
+  <si>
+    <t>TC_CART_07</t>
+  </si>
+  <si>
+    <t>TC_CART_08</t>
+  </si>
+  <si>
+    <t>TC_CART_09</t>
+  </si>
+  <si>
+    <t>TC_CART_10</t>
+  </si>
+  <si>
+    <t>Verify functionality of remove button</t>
+  </si>
+  <si>
+    <t>System should remove the item from cart on remove button action</t>
+  </si>
+  <si>
+    <t>Verify functionality of Continue shopping button</t>
+  </si>
+  <si>
+    <t>System should redirect user to product page on continue shopping button action</t>
+  </si>
+  <si>
+    <t>Verify functionality of Checkout button</t>
+  </si>
+  <si>
+    <t>Verify functionality of Checkout button on empty cart</t>
+  </si>
+  <si>
+    <t>System should show four options (All items, About, Logout and Reset App State)</t>
+  </si>
+  <si>
+    <t>Verify cart number behaviour</t>
+  </si>
+  <si>
+    <t>Cart icon number should be increase decrease on the action of add/remove respectively</t>
+  </si>
+  <si>
+    <t>Verify product name</t>
+  </si>
+  <si>
+    <t>Verify product description</t>
+  </si>
+  <si>
+    <t>System should show the correct product name as on product page</t>
+  </si>
+  <si>
+    <t>System should show the correct product description as on product page</t>
+  </si>
+  <si>
+    <t>TC_CART_11</t>
+  </si>
+  <si>
+    <t>TC_CART_12</t>
+  </si>
+  <si>
+    <t>TC_CART_13</t>
+  </si>
+  <si>
+    <t>TC_CART_14</t>
+  </si>
+  <si>
+    <t>TC_CART_15</t>
+  </si>
+  <si>
+    <t>Verify product price</t>
+  </si>
+  <si>
+    <t>System should show the correct product price as on product page</t>
+  </si>
+  <si>
+    <t>Verify product redirection through name</t>
+  </si>
+  <si>
+    <t>System should redirect user to product page on click product name</t>
+  </si>
+  <si>
+    <t>Verify footer user interface</t>
+  </si>
+  <si>
+    <t>Footer section and content should clear and visible clearly without any ui mismatch</t>
+  </si>
+  <si>
+    <t>Verify footer redirection</t>
+  </si>
+  <si>
+    <t>System should redirect user to correct social media page</t>
+  </si>
+  <si>
+    <t>TC_CART_16</t>
+  </si>
+  <si>
+    <t>System should redirect user to checkout information page even when cart is empty</t>
+  </si>
+  <si>
+    <t>Verify cart page when no any item added</t>
+  </si>
+  <si>
+    <t>System should show the cart page even when no any item added</t>
+  </si>
+  <si>
+    <t>Verify quantity of added products</t>
+  </si>
+  <si>
+    <t>Quantity column should displayed "1" for each item added</t>
+  </si>
+  <si>
+    <t>System should redirect user to checkout information page on checkout button action</t>
+  </si>
+  <si>
+    <t>System should show each added product</t>
+  </si>
+  <si>
+    <t>TC_CART_17</t>
+  </si>
+  <si>
+    <t>Cart items should be present after refresh</t>
+  </si>
+  <si>
+    <t>TC_CART_18</t>
+  </si>
+  <si>
+    <t>Verify cart persists after page refresh</t>
+  </si>
+  <si>
+    <t>Verify cart persists after logout/login</t>
+  </si>
+  <si>
+    <t>System should persists cart after logout and login</t>
+  </si>
+  <si>
+    <t>TC_CART_19</t>
+  </si>
+  <si>
+    <t>Verify cart icon clickable</t>
+  </si>
+  <si>
+    <t>Cart icon should be clickable</t>
+  </si>
+  <si>
+    <t>Verify functionality of navbar hamburger button</t>
+  </si>
+  <si>
+    <t>1.Open saucedemo website
+2.Login with valid credential
+3.Click the navbar hamburger button of product page
+4.Click logout option
+4.Observe the redirected page</t>
+  </si>
+  <si>
+    <t>Pre-Condition</t>
+  </si>
+  <si>
+    <t>User should be login and present on item page</t>
+  </si>
+  <si>
+    <t>1.Add some item to cart
+2.Go to cart module
+3.Verify the added items</t>
+  </si>
+  <si>
+    <t>1.Add some item to cart
+2.Go to cart module
+3.Observe the cart page</t>
+  </si>
+  <si>
+    <t>1.Add some item to cart
+2.Go to cart module
+3.Click the remove button of any item
+4.Verify the item is removed from cart</t>
+  </si>
+  <si>
+    <t>1.Add some item to cart
+2.Go to cart module
+3.Click the continue shopping button
+4.Verify user is redirected to product page</t>
+  </si>
+  <si>
+    <t>1.Add some item to cart
+2.Go to cart module
+3.Click the checkout button
+4.Verify user is redirected to checkout information page</t>
+  </si>
+  <si>
+    <t>1.Go to cart module without adding any item
+2.Click checkout
+3.Verify user is redirected to checkout information page</t>
+  </si>
+  <si>
+    <t>1.Go to cart
+2.Click the navbar hamburger button
+3.Verify 4 options should be displayed</t>
+  </si>
+  <si>
+    <t>1.Add 2 items
+2.Go to cart
+3.Click remove button of first item
+4.Verify from the cart icon number</t>
+  </si>
+  <si>
+    <t>1.Add 1 product to cart
+2.Go to cart
+3.Verify from the product name</t>
+  </si>
+  <si>
+    <t>1.Add 1 product to cart
+2.Go to cart
+3.Verify from the product description</t>
+  </si>
+  <si>
+    <t>1.Add 1 product to cart
+2.Go to cart
+3.Verify from the product price</t>
+  </si>
+  <si>
+    <t>1.Add 1 product to cart
+2.Go to cart
+3.Click the product name
+4.Verify by the redirected page</t>
+  </si>
+  <si>
+    <t>1.Go to cart
+2.Observe the footer</t>
+  </si>
+  <si>
+    <t>1.Go to cart
+2.Click any social media icon in footer
+3.Verify from the redirected media page</t>
+  </si>
+  <si>
+    <t>1.Go to cart without adding any item
+2.Observe the cart page</t>
+  </si>
+  <si>
+    <t>1.Add an item to cart
+2.Go to cart
+3.Verify the quantity of added item</t>
+  </si>
+  <si>
+    <t>1.Add 2 item to cart
+2.Go to cart
+3.Refresh page
+4.Verify all the items still present</t>
+  </si>
+  <si>
+    <t>1.Add any item to cart
+2.Logout from the account
+3.Login again with standard user credential
+4.Verify the added item in cart</t>
+  </si>
+  <si>
+    <t>1.Verify cart icon clickable</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_01</t>
+  </si>
+  <si>
+    <t>Verify correct number of items displayed during checkout</t>
+  </si>
+  <si>
+    <t>User logged in and item added to cart</t>
+  </si>
+  <si>
+    <t>Cart icon should display correct number of items</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_02</t>
+  </si>
+  <si>
+    <t>Verify user can access checkout page with 0,1 or multiple items</t>
+  </si>
+  <si>
+    <t>User logged in</t>
+  </si>
+  <si>
+    <t>System should open Checkout Your Information page</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_03</t>
+  </si>
+  <si>
+    <t>Verify cancel button redirects to cart page</t>
+  </si>
+  <si>
+    <t>User on Checkout Information page</t>
+  </si>
+  <si>
+    <t>1. Click Cancel button</t>
+  </si>
+  <si>
+    <t>User should be redirected to cart page</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_04</t>
+  </si>
+  <si>
+    <t>Verify continue button with valid input</t>
+  </si>
+  <si>
+    <t>User should be redirected to Checkout Overview page</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_05</t>
+  </si>
+  <si>
+    <t>Verify hamburger menu options</t>
+  </si>
+  <si>
+    <t>1. Click hamburger menu icon</t>
+  </si>
+  <si>
+    <t>Menu should show All Items, About, Logout and Reset App State options</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_06</t>
+  </si>
+  <si>
+    <t>Verify All Items option redirection</t>
+  </si>
+  <si>
+    <t>User should be redirected to Products page</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_07</t>
+  </si>
+  <si>
+    <t>Verify Logout functionality</t>
+  </si>
+  <si>
+    <t>User should be redirected to login page</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_08</t>
+  </si>
+  <si>
+    <t>Verify About page redirection</t>
+  </si>
+  <si>
+    <t>User should be redirected to SauceDemo About page</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_09</t>
+  </si>
+  <si>
+    <t>Verify Reset App State resets cart items</t>
+  </si>
+  <si>
+    <t>User logged in with items in cart</t>
+  </si>
+  <si>
+    <t>Cart item count should become 0</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_10</t>
+  </si>
+  <si>
+    <t>Verify Swag Labs brand name visibility</t>
+  </si>
+  <si>
+    <t>1. Observe header</t>
+  </si>
+  <si>
+    <t>Swag Labs brand name should be visible</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_11</t>
+  </si>
+  <si>
+    <t>Verify Checkout Your Information label visibility</t>
+  </si>
+  <si>
+    <t>1. Observe page title</t>
+  </si>
+  <si>
+    <t>Checkout: Your Information label should be visible</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_12</t>
+  </si>
+  <si>
+    <t>Verify cart icon visibility</t>
+  </si>
+  <si>
+    <t>1. Observe cart icon</t>
+  </si>
+  <si>
+    <t>Cart icon and item count should be visible</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_13</t>
+  </si>
+  <si>
+    <t>Verify input fields visibility</t>
+  </si>
+  <si>
+    <t>1. Observe input fields</t>
+  </si>
+  <si>
+    <t>First Name, Last Name and Postal Code fields should be visible</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_14</t>
+  </si>
+  <si>
+    <t>Verify user can enter data in input fields</t>
+  </si>
+  <si>
+    <t>1. Enter values in all fields</t>
+  </si>
+  <si>
+    <t>User should be able to enter data successfully</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_15</t>
+  </si>
+  <si>
+    <t>Verify system behaviour on invalid/blank input</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_16</t>
+  </si>
+  <si>
+    <t>Verify error message for blank First Name</t>
+  </si>
+  <si>
+    <t>Error message "First Name is required" should appear</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_17</t>
+  </si>
+  <si>
+    <t>Verify error message for blank Last Name</t>
+  </si>
+  <si>
+    <t>Error message "Last Name is required" should appear</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_18</t>
+  </si>
+  <si>
+    <t>Verify error message for blank Postal Code</t>
+  </si>
+  <si>
+    <t>Error message "Postal Code is required" should appear</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_19</t>
+  </si>
+  <si>
+    <t>Verify footer visibility</t>
+  </si>
+  <si>
+    <t>1. Scroll to footer</t>
+  </si>
+  <si>
+    <t>Footer content should be clearly visible</t>
+  </si>
+  <si>
+    <t>TC_CHECKOUT_20</t>
+  </si>
+  <si>
+    <t>Verify footer social media links</t>
+  </si>
+  <si>
+    <t>1. Click social media icon in footer</t>
+  </si>
+  <si>
+    <t>User should be redirected to correct social media page</t>
+  </si>
+  <si>
+    <t>1. Go to cart 
+2. Click Checkout 
+3. Observe cart icon number</t>
+  </si>
+  <si>
+    <t>1. Go to cart with 0 items 
+2. Click Checkout 
+3. Repeat with 1 item and multiple items</t>
+  </si>
+  <si>
+    <t>1. Enter First Name 
+2. Enter Last Name 
+3. Enter Postal Code 
+4. Click Continue</t>
+  </si>
+  <si>
+    <t>First Name: John Last Name: Doe 
+Postal Code: 400001</t>
+  </si>
+  <si>
+    <t>1. Open hamburger menu 
+2. Click All Items</t>
+  </si>
+  <si>
+    <t>1. Open hamburger menu 
+2. Click Logout</t>
+  </si>
+  <si>
+    <t>1. Open hamburger menu 
+2. Click About</t>
+  </si>
+  <si>
+    <t>1. Add item to cart 
+2. Open hamburger menu 
+3. Click Reset App State</t>
+  </si>
+  <si>
+    <t>First Name: John 
+Last Name: Doe 
+Postal Code: 400001</t>
+  </si>
+  <si>
+    <t>1. Leave fields blank 
+2. Click Continue</t>
+  </si>
+  <si>
+    <t>System should redirect user to checkout overview page</t>
+  </si>
+  <si>
+    <t>First Name: "   " 
+Last Name: "    "
+Postal Code: "      "</t>
+  </si>
+  <si>
+    <t>1. Leave First Name blank 
+2. Enter other fields 
+3. Click Continue</t>
+  </si>
+  <si>
+    <t>Last Name: Doe 
+Postal Code: 400001</t>
+  </si>
+  <si>
+    <t>1. Enter First Name 
+2. Leave Last Name blank 
+3. Click Continue</t>
+  </si>
+  <si>
+    <t>First Name: John 
+Postal Code: 400001</t>
+  </si>
+  <si>
+    <t>1. Enter First Name 
+2. Enter Last Name 
+3. Leave Postal Code blank 4. Click Continue</t>
+  </si>
+  <si>
+    <t>First Name: John 
+Last Name: Doe</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_01</t>
+  </si>
+  <si>
+    <t>User logged in and items added to cart</t>
+  </si>
+  <si>
+    <t>1. Add items to cart_x000D_
+2. Go to cart_x000D_
+3. Click Checkout_x000D_
+4. Fill checkout information_x000D_
+5. Observe cart icon number on Overview page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_02</t>
+  </si>
+  <si>
+    <t>Verify user can access checkout overview page with 0,1 or multiple items</t>
+  </si>
+  <si>
+    <t>1. Go to cart with 0 items_x000D_
+2. Click Checkout_x000D_
+3. Repeat with 1 item and multiple items_x000D_
+4. Complete checkout information</t>
+  </si>
+  <si>
+    <t>System should open Checkout: Overview page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_03</t>
+  </si>
+  <si>
+    <t>Verify cancel button redirects to products page</t>
+  </si>
+  <si>
+    <t>User on Checkout Overview page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_04</t>
+  </si>
+  <si>
+    <t>Verify finish button redirects to complete page</t>
+  </si>
+  <si>
+    <t>1. Click Finish button</t>
+  </si>
+  <si>
+    <t>User should be redirected to Checkout Complete page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_05</t>
+  </si>
+  <si>
+    <t>Verify cart icon navigation</t>
+  </si>
+  <si>
+    <t>1. Click cart icon</t>
+  </si>
+  <si>
+    <t>User should be redirected to Cart page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_06</t>
+  </si>
+  <si>
+    <t>Verify navbar hamburger menu options</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_07</t>
+  </si>
+  <si>
+    <t>1. Open hamburger menu_x000D_
+2. Click All Items</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_08</t>
+  </si>
+  <si>
+    <t>1. Open hamburger menu_x000D_
+2. Click Logout</t>
+  </si>
+  <si>
+    <t>User should be redirected to Login page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_09</t>
+  </si>
+  <si>
+    <t>1. Open hamburger menu_x000D_
+2. Click About</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_10</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_11</t>
+  </si>
+  <si>
+    <t>Verify Checkout Overview label visibility</t>
+  </si>
+  <si>
+    <t>Checkout: Overview label should be visible</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_12</t>
+  </si>
+  <si>
+    <t>Verify quantity and description label visibility</t>
+  </si>
+  <si>
+    <t>1. Observe QTY and Description labels</t>
+  </si>
+  <si>
+    <t>QTY and Description labels should be clearly visible</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_13</t>
+  </si>
+  <si>
+    <t>Verify quantity displayed correctly</t>
+  </si>
+  <si>
+    <t>1. Add item to cart_x000D_
+2. Go to checkout overview_x000D_
+3. Observe quantity column</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_14</t>
+  </si>
+  <si>
+    <t>Verify correct item name displayed</t>
+  </si>
+  <si>
+    <t>1. Observe item name in product list</t>
+  </si>
+  <si>
+    <t>Item name should match the product added to cart</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_15</t>
+  </si>
+  <si>
+    <t>Verify product name redirection</t>
+  </si>
+  <si>
+    <t>1. Click product name</t>
+  </si>
+  <si>
+    <t>User should be redirected to product details page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_16</t>
+  </si>
+  <si>
+    <t>Verify correct product description</t>
+  </si>
+  <si>
+    <t>1. Observe product description</t>
+  </si>
+  <si>
+    <t>Product description should match product page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_17</t>
+  </si>
+  <si>
+    <t>Verify correct product price</t>
+  </si>
+  <si>
+    <t>1. Observe product price</t>
+  </si>
+  <si>
+    <t>Product price should match product page</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_18</t>
+  </si>
+  <si>
+    <t>Verify payment information visibility</t>
+  </si>
+  <si>
+    <t>1. Observe payment information section</t>
+  </si>
+  <si>
+    <t>Payment information should be displayed correctly</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_19</t>
+  </si>
+  <si>
+    <t>Verify shipping information visibility</t>
+  </si>
+  <si>
+    <t>1. Observe shipping information section</t>
+  </si>
+  <si>
+    <t>Shipping information should be displayed correctly</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_20</t>
+  </si>
+  <si>
+    <t>Verify item total calculation</t>
+  </si>
+  <si>
+    <t>1. Note product prices_x000D_
+2. Calculate total_x000D_
+3. Compare with item total displayed</t>
+  </si>
+  <si>
+    <t>Item total should equal sum of product prices</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_21</t>
+  </si>
+  <si>
+    <t>Verify final total calculation</t>
+  </si>
+  <si>
+    <t>1. Note item total_x000D_
+2. Add tax_x000D_
+3. Compare with displayed total</t>
+  </si>
+  <si>
+    <t>Final total should equal item total + tax</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_22</t>
+  </si>
+  <si>
+    <t>TC_OVERVIEW_23</t>
+  </si>
+  <si>
+    <t>Quantity value should be 1 for each item</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_01</t>
+  </si>
+  <si>
+    <t>1.User is on checkout complete page</t>
+  </si>
+  <si>
+    <t>1.Observe the cart icon</t>
+  </si>
+  <si>
+    <t>Username : standard_user
+Password : secret_sauce
+First Name: John
+Last Name: Doe
+Pstal Code: 400001</t>
+  </si>
+  <si>
+    <t>Username : standard_user
+Password : secret_sauce
+First Name: John
+Last Name: Doe
+Pstal Code: 400002</t>
+  </si>
+  <si>
+    <t>Username : standard_user
+Password : secret_sauce
+First Name: John
+Last Name: Doe
+Pstal Code: 400003</t>
+  </si>
+  <si>
+    <t>Verify cart icon status</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_02</t>
+  </si>
+  <si>
+    <t>Verify cart is empty</t>
+  </si>
+  <si>
+    <t>1.Click the cart button
+2.Observe the cart page</t>
+  </si>
+  <si>
+    <t>Cart page should be empty</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_03</t>
+  </si>
+  <si>
+    <t>Verify user redirects to all item page</t>
+  </si>
+  <si>
+    <t>1.Click back home button
+2.Observe the redirected page
+3.Observe the item add to cart button</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_04</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_05</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_06</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_07</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_08</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_09</t>
+  </si>
+  <si>
+    <t>Verify Checkout Complete label visibility</t>
+  </si>
+  <si>
+    <t>Checkout: Complete label should be visible</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_10</t>
+  </si>
+  <si>
+    <t>Verify successful image visibility</t>
+  </si>
+  <si>
+    <t>1.Observe the green tick successful image</t>
+  </si>
+  <si>
+    <t>Green tick successful image should be visible to user</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_11</t>
+  </si>
+  <si>
+    <t>Verify thank you message</t>
+  </si>
+  <si>
+    <t>1.Verify thank you message</t>
+  </si>
+  <si>
+    <t>System should show thank you message "Thank you for your order!
+Your order has been dispatched, and will arrive just as fast as the pony can get there!"</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_12</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_13</t>
+  </si>
+  <si>
+    <t>TC_COMPLETE_14</t>
+  </si>
+  <si>
+    <t>Verify page refresh function</t>
+  </si>
+  <si>
+    <t>1.Refresh the page</t>
+  </si>
+  <si>
+    <t>User should still present on complete page after refresh</t>
+  </si>
+  <si>
+    <t>User should be redirected to all item page and add to cart button should be available for each item</t>
+  </si>
+  <si>
+    <t>Cart icon should not display item count after order completion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -556,6 +1495,12 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -602,12 +1547,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1264,8 +2215,8 @@
   <cols>
     <col min="1" max="1" width="18.109375" customWidth="1"/>
     <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.5546875" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -1293,7 +2244,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>77</v>
       </c>
@@ -1304,7 +2255,7 @@
         <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>81</v>
@@ -1323,7 +2274,7 @@
         <v>83</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>108</v>
@@ -1342,7 +2293,7 @@
         <v>79</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>86</v>
@@ -1350,7 +2301,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>88</v>
       </c>
@@ -1361,15 +2312,15 @@
         <v>79</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>90</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>91</v>
       </c>
@@ -1380,15 +2331,15 @@
         <v>79</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>93</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>94</v>
       </c>
@@ -1399,15 +2350,15 @@
         <v>96</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>97</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>98</v>
       </c>
@@ -1418,15 +2369,15 @@
         <v>100</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>97</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>101</v>
       </c>
@@ -1437,15 +2388,15 @@
         <v>103</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>104</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>105</v>
       </c>
@@ -1456,15 +2407,15 @@
         <v>110</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>107</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>109</v>
       </c>
@@ -1475,15 +2426,15 @@
         <v>111</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>112</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>113</v>
       </c>
@@ -1494,15 +2445,15 @@
         <v>115</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>116</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>117</v>
       </c>
@@ -1513,15 +2464,15 @@
         <v>118</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>119</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>120</v>
       </c>
@@ -1532,15 +2483,15 @@
         <v>121</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>122</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" ht="156" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>123</v>
       </c>
@@ -1548,51 +2499,51 @@
         <v>124</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>126</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="78" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>130</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>134</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1607,10 +2558,18 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="26.109375" customWidth="1"/>
+    <col min="4" max="4" width="26.5546875" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="6" max="6" width="32.88671875" customWidth="1"/>
+    <col min="7" max="7" width="28.109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1618,22 +2577,444 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
+    <row r="2" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" ht="109.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1643,33 +3024,1400 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.88671875" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" customWidth="1"/>
+    <col min="5" max="5" width="25.77734375" customWidth="1"/>
+    <col min="6" max="6" width="23.33203125" customWidth="1"/>
+    <col min="7" max="7" width="21.77734375" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
+    </row>
+    <row r="2" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{591D7AD8-0D17-45C3-9B20-FC626F8000A1}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="3" max="3" width="28.109375" customWidth="1"/>
+    <col min="4" max="4" width="39.5546875" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+    </row>
+    <row r="3" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+    </row>
+    <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+    </row>
+    <row r="5" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+    </row>
+    <row r="17" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+    </row>
+    <row r="23" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E91ED0A1-856D-42DA-94C8-149A2BF82238}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="27.44140625" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.44140625" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" customWidth="1"/>
+    <col min="6" max="6" width="35.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>